<commit_message>
Include contact email in exports and imports
</commit_message>
<xml_diff>
--- a/test-data/imports/explicit_clearing.xlsx
+++ b/test-data/imports/explicit_clearing.xlsx
@@ -1,92 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="csv_example (2).csv" sheetId="1" r:id="rId4"/>
+    <sheet name="csv_example (2).csv" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
-  <si>
-    <t>URN:Tel</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>language</t>
-  </si>
-  <si>
-    <t>Created On</t>
-  </si>
-  <si>
-    <t xml:space="preserve">field: goats </t>
-  </si>
-  <si>
-    <t>Field:Sheep</t>
-  </si>
-  <si>
-    <t>+250788123123</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>eng</t>
-  </si>
-  <si>
-    <t>+250788456456</t>
-  </si>
-  <si>
-    <t>Mary Smith</t>
-  </si>
-  <si>
-    <t>spa</t>
-  </si>
-  <si>
-    <t>+250788456678</t>
-  </si>
-  <si>
-    <t>--</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> -- </t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="0" formatCode="General"/>
-    <numFmt numFmtId="59" formatCode="d mmm yyyy"/>
-    <numFmt numFmtId="60" formatCode="d/m/yyyy"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="d mmm yyyy"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
   <fonts count="3">
     <font>
+      <name val="Calibri"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color indexed="8"/>
       <sz val="12"/>
-      <color indexed="8"/>
-      <name val="Helvetica Neue"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color indexed="8"/>
       <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -123,38 +74,44 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="60" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="ff000000"/>
@@ -1258,151 +1215,209 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="10.8333" defaultRowHeight="16" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="10.8333" defaultRowHeight="16" customHeight="1" outlineLevelRow="0"/>
   <cols>
-    <col min="1" max="1" width="24.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="21" style="1" customWidth="1"/>
-    <col min="3" max="4" width="12.3516" style="1" customWidth="1"/>
-    <col min="5" max="5" width="10.8516" style="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="10.8516" style="1" customWidth="1"/>
+    <col width="24.5" customWidth="1" style="1" min="1" max="1"/>
+    <col width="21" customWidth="1" style="1" min="2" max="2"/>
+    <col width="12.3516" customWidth="1" style="1" min="3" max="4"/>
+    <col width="10.8516" customWidth="1" style="1" min="5" max="5"/>
+    <col width="10.5" customWidth="1" style="1" min="6" max="6"/>
+    <col width="10.8516" customWidth="1" style="1" min="7" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.35" customHeight="1">
-      <c r="A1" t="s" s="2">
+    <row r="1" ht="15.35" customHeight="1" s="7">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>URN:Tel</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Created On</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">field: goats </t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Field:Sheep</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.35" customHeight="1" s="7">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>+250788123123</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>John Doe</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>eng</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>44091</v>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="2">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="2">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s" s="2">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>john@doe.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15.35" customHeight="1" s="7">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>+250788456456</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Mary Smith</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>spa</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>43961</v>
+      </c>
+      <c r="E3" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="2">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="2">
+      <c r="F3" s="6" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="2" ht="15.35" customHeight="1">
-      <c r="A2" t="s" s="2">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s" s="2">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s" s="2">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3">
-        <v>44091</v>
-      </c>
-      <c r="E2" s="4">
-        <v>1</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0</v>
+    <row r="4" ht="15.35" customHeight="1" s="7">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>+250788456678</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>43993</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> -- </t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>--</t>
+        </is>
       </c>
     </row>
-    <row r="3" ht="15.35" customHeight="1">
-      <c r="A3" t="s" s="2">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s" s="2">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s" s="2">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5">
-        <v>43961</v>
-      </c>
-      <c r="E3" s="4">
-        <v>3</v>
-      </c>
-      <c r="F3" s="4">
-        <v>5</v>
-      </c>
+    <row r="5" ht="15.35" customHeight="1" s="7">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
     </row>
-    <row r="4" ht="15.35" customHeight="1">
-      <c r="A4" t="s" s="2">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D4" s="5">
-        <v>43993</v>
-      </c>
-      <c r="E4" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s" s="2">
-        <v>13</v>
-      </c>
+    <row r="6" ht="15.35" customHeight="1" s="7">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
     </row>
-    <row r="5" ht="15.35" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+    <row r="7" ht="15.35" customHeight="1" s="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
     </row>
-    <row r="6" ht="15.35" customHeight="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+    <row r="8" ht="15.35" customHeight="1" s="7">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
     </row>
-    <row r="7" ht="15.35" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
+    <row r="9" ht="15.35" customHeight="1" s="7">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
     </row>
-    <row r="8" ht="15.35" customHeight="1">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-    </row>
-    <row r="9" ht="15.35" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" ht="15.35" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+    <row r="10" ht="15.35" customHeight="1" s="7">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="0" pageOrder="downThenOver"/>
   <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12 &amp;K000000&amp;P</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>